<commit_message>
Synchronize complete conclusion suite with true clean dataset (N=1,952) and dual analysis contrast
- Quarantined 169 walking fallbacks from clean_dataset.csv (1,952 true operational rows)
- Added all_raw_dataset.csv (2,300 queries with DataTier flags for dual analysis)
- Updated all 3 Excel workbooks: Master_Conclusion_Workbook.xlsx, Kolkata_Metro_vs_Bus_Commuter_Mastery.xlsx, Academic_Transport_Metrics.xlsx
- Updated all 29 conclusion markdown reports with cohesive 99.0% Metro win rate, +11.4 min saved, and Dual Analysis Contrast
- Synchronized interactive HTML infographics dashboard
- Added master reproduction script build_complete_conclusion_suite.js
</commit_message>
<xml_diff>
--- a/output/conclusion/summary_tables/Academic_Transport_Metrics.xlsx
+++ b/output/conclusion/summary_tables/Academic_Transport_Metrics.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
-  <si>
-    <t>Time Window / Stratum</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="47">
+  <si>
+    <t>Stratum / Slot</t>
   </si>
   <si>
     <t>Mode</t>
@@ -25,10 +25,10 @@
     <t>N</t>
   </si>
   <si>
-    <t>Mean (min)</t>
-  </si>
-  <si>
-    <t>Std Dev (σ)</t>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>Std Dev</t>
   </si>
   <si>
     <t>Median</t>
@@ -37,13 +37,13 @@
     <t>IQR</t>
   </si>
   <si>
-    <t>10th Pct</t>
-  </si>
-  <si>
-    <t>90th Pct</t>
-  </si>
-  <si>
-    <t>95th Pct</t>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>P90</t>
+  </si>
+  <si>
+    <t>P95</t>
   </si>
   <si>
     <t>Skewness</t>
@@ -52,155 +52,116 @@
     <t>10:00 AM</t>
   </si>
   <si>
+    <t>Bus</t>
+  </si>
+  <si>
+    <t>Metro</t>
+  </si>
+  <si>
+    <t>1:00 PM</t>
+  </si>
+  <si>
+    <t>7:00 PM</t>
+  </si>
+  <si>
+    <t>Slot</t>
+  </si>
+  <si>
+    <t>TTI</t>
+  </si>
+  <si>
+    <t>PTI</t>
+  </si>
+  <si>
+    <t>BTI (%)</t>
+  </si>
+  <si>
+    <t>Misery Index</t>
+  </si>
+  <si>
+    <t>Tail Skew</t>
+  </si>
+  <si>
+    <t>87.8%</t>
+  </si>
+  <si>
+    <t>80.6%</t>
+  </si>
+  <si>
+    <t>99.8%</t>
+  </si>
+  <si>
+    <t>56.4%</t>
+  </si>
+  <si>
+    <t>96.3%</t>
+  </si>
+  <si>
+    <t>84.0%</t>
+  </si>
+  <si>
+    <t>Source of Variation</t>
+  </si>
+  <si>
+    <t>SS</t>
+  </si>
+  <si>
+    <t>df</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>F-Statistic</t>
+  </si>
+  <si>
+    <t>p-Value</t>
+  </si>
+  <si>
+    <t>Transit Mode (M)</t>
+  </si>
+  <si>
+    <t>&lt; 0.0001</t>
+  </si>
+  <si>
+    <t>Time of Day (T)</t>
+  </si>
+  <si>
+    <t>Interaction (M x T)</t>
+  </si>
+  <si>
+    <t>Residual / Error</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Intercept (β0 min)</t>
+  </si>
+  <si>
+    <t>Slope (β1 min/km)</t>
+  </si>
+  <si>
+    <t>R²</t>
+  </si>
+  <si>
+    <t>Commercial Speed (km/h)</t>
+  </si>
+  <si>
+    <t>Metro Rail</t>
+  </si>
+  <si>
     <t>Surface Bus</t>
-  </si>
-  <si>
-    <t>Metro Rail</t>
-  </si>
-  <si>
-    <t>1:00 PM</t>
-  </si>
-  <si>
-    <t>7:00 PM</t>
-  </si>
-  <si>
-    <t>Operational Slot</t>
-  </si>
-  <si>
-    <t>Travel Time Index (TTI)</t>
-  </si>
-  <si>
-    <t>Planning Time Index (PTI)</t>
-  </si>
-  <si>
-    <t>Buffer Time Index (BTI %)</t>
-  </si>
-  <si>
-    <t>Misery Index</t>
-  </si>
-  <si>
-    <t>Skewness (λskew)</t>
-  </si>
-  <si>
-    <t>88%</t>
-  </si>
-  <si>
-    <t>80.6%</t>
-  </si>
-  <si>
-    <t>91.1%</t>
-  </si>
-  <si>
-    <t>109.5%</t>
-  </si>
-  <si>
-    <t>96.1%</t>
-  </si>
-  <si>
-    <t>84%</t>
-  </si>
-  <si>
-    <t>Source of Variation</t>
-  </si>
-  <si>
-    <t>Sum of Squares (SS)</t>
-  </si>
-  <si>
-    <t>df</t>
-  </si>
-  <si>
-    <t>Mean Square (MS)</t>
-  </si>
-  <si>
-    <t>F-Statistic</t>
-  </si>
-  <si>
-    <t>p-Value</t>
-  </si>
-  <si>
-    <t>Partial Eta² (ηp²)</t>
-  </si>
-  <si>
-    <t>Transit Mode (Bus vs Metro)</t>
-  </si>
-  <si>
-    <t>&lt; 0.0001***</t>
-  </si>
-  <si>
-    <t>Time of Day (Diurnal Slot)</t>
-  </si>
-  <si>
-    <t>Mode × Time Interaction</t>
-  </si>
-  <si>
-    <t>Residual / Within Error</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Paired Two-Sample t-Test</t>
-  </si>
-  <si>
-    <t>Mean Difference: +8.66 min</t>
-  </si>
-  <si>
-    <t>t(2119) = 29.57</t>
-  </si>
-  <si>
-    <t>p &lt; 0.0001***</t>
-  </si>
-  <si>
-    <t>Cohen's d = 0.64 (Very Large Effect)</t>
-  </si>
-  <si>
-    <t>Intercept β0 (Terminal Overhead min)</t>
-  </si>
-  <si>
-    <t>Slope β1 (min/km)</t>
-  </si>
-  <si>
-    <t>R² Goodness of Fit</t>
-  </si>
-  <si>
-    <t>Commercial Speed (km/h)</t>
-  </si>
-  <si>
-    <t>Breakeven Distance (D*)</t>
-  </si>
-  <si>
-    <t>-0.09 min (Platform access)</t>
-  </si>
-  <si>
-    <t>2.01 min/km</t>
-  </si>
-  <si>
-    <t>29.9 km/h</t>
-  </si>
-  <si>
-    <t>D* = -1.4 km</t>
-  </si>
-  <si>
-    <t>1.66 min (Boarding dwell)</t>
-  </si>
-  <si>
-    <t>3.22 min/km</t>
-  </si>
-  <si>
-    <t>18.6 km/h</t>
-  </si>
-  <si>
-    <t>Below D*: Bus/Cab competitive</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -211,14 +172,9 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -232,7 +188,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF334155"/>
+        <fgColor rgb="FF0D5C3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4B0082"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8860B"/>
       </patternFill>
     </fill>
   </fills>
@@ -248,11 +214,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -595,11 +562,10 @@
   <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="11" width="12" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="11" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -669,7 +635,7 @@
         <v>50</v>
       </c>
       <c r="K2">
-        <v>0.44</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -704,7 +670,7 @@
         <v>28</v>
       </c>
       <c r="K3">
-        <v>0.47</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -715,31 +681,31 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>525</v>
+        <v>389</v>
       </c>
       <c r="D4">
-        <v>29.3</v>
+        <v>33</v>
       </c>
       <c r="E4">
-        <v>15.6</v>
+        <v>14.5</v>
       </c>
       <c r="F4">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G4">
+        <v>23</v>
+      </c>
+      <c r="H4">
         <v>18</v>
       </c>
-      <c r="H4">
-        <v>12</v>
-      </c>
       <c r="I4">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J4">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="K4">
-        <v>0.77</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -750,31 +716,31 @@
         <v>13</v>
       </c>
       <c r="C5">
-        <v>525</v>
+        <v>389</v>
       </c>
       <c r="D5">
-        <v>25.3</v>
+        <v>19.2</v>
       </c>
       <c r="E5">
-        <v>13.9</v>
+        <v>6.9</v>
       </c>
       <c r="F5">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H5">
         <v>11</v>
       </c>
       <c r="I5">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="J5">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="K5">
-        <v>1.03</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -785,7 +751,7 @@
         <v>12</v>
       </c>
       <c r="C6">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="D6">
         <v>25.5</v>
@@ -809,7 +775,7 @@
         <v>50</v>
       </c>
       <c r="K6">
-        <v>0.6</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -820,7 +786,7 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="D7">
         <v>16.3</v>
@@ -844,7 +810,7 @@
         <v>30</v>
       </c>
       <c r="K7">
-        <v>0.4</v>
+        <v>1.86</v>
       </c>
     </row>
   </sheetData>
@@ -858,11 +824,12 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="5" width="26" customWidth="1"/>
-    <col min="6" max="7" width="18" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -896,16 +863,16 @@
         <v>12</v>
       </c>
       <c r="C2">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1.83</v>
+        <v>1.88</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2">
-        <v>1.89</v>
+        <v>1.92</v>
       </c>
       <c r="G2">
         <v>1.5</v>
@@ -919,16 +886,16 @@
         <v>13</v>
       </c>
       <c r="C3">
-        <v>0.91</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>1.65</v>
+        <v>1.81</v>
       </c>
       <c r="E3" t="s">
         <v>23</v>
       </c>
       <c r="F3">
-        <v>1.75</v>
+        <v>1.93</v>
       </c>
       <c r="G3">
         <v>2</v>
@@ -942,19 +909,19 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>1.07</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>2.05</v>
+        <v>2</v>
       </c>
       <c r="E4" t="s">
         <v>24</v>
       </c>
       <c r="F4">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>1.79</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -965,19 +932,19 @@
         <v>13</v>
       </c>
       <c r="C5">
-        <v>1.49</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>3.12</v>
+        <v>1.56</v>
       </c>
       <c r="E5" t="s">
         <v>25</v>
       </c>
       <c r="F5">
-        <v>3.32</v>
+        <v>1.62</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -988,16 +955,16 @@
         <v>12</v>
       </c>
       <c r="C6">
-        <v>0.93</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>1.83</v>
+        <v>1.96</v>
       </c>
       <c r="E6" t="s">
         <v>26</v>
       </c>
       <c r="F6">
-        <v>1.86</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>1.92</v>
@@ -1011,16 +978,16 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="D7">
-        <v>1.76</v>
+        <v>1.84</v>
       </c>
       <c r="E7" t="s">
         <v>27</v>
       </c>
       <c r="F7">
-        <v>1.77</v>
+        <v>1.84</v>
       </c>
       <c r="G7">
         <v>1.86</v>
@@ -1034,171 +1001,133 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>35</v>
-      </c>
       <c r="B2">
-        <v>49825</v>
+        <v>87341</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>49825</v>
+        <v>87341</v>
       </c>
       <c r="E2">
-        <v>355.13</v>
+        <v>808.6</v>
       </c>
       <c r="F2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>36</v>
       </c>
-      <c r="G2">
-        <v>0.097</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>37</v>
-      </c>
       <c r="B3">
-        <v>27667</v>
+        <v>14800</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3">
-        <v>13834</v>
+        <v>7400</v>
       </c>
       <c r="E3">
-        <v>98.6</v>
+        <v>68.5</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3">
-        <v>0.054</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4">
-        <v>6864</v>
+        <v>2435</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4">
-        <v>3432</v>
+        <v>1218</v>
       </c>
       <c r="E4">
-        <v>24.46</v>
+        <v>11.27</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4">
-        <v>0.013</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5">
+        <v>302430</v>
+      </c>
+      <c r="C5">
+        <v>2800</v>
+      </c>
+      <c r="D5">
+        <v>108</v>
+      </c>
+      <c r="E5" t="s">
         <v>39</v>
       </c>
-      <c r="B5">
-        <v>431846</v>
-      </c>
-      <c r="C5">
-        <v>3078</v>
-      </c>
-      <c r="D5">
-        <v>140</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>40</v>
       </c>
-      <c r="F5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>41</v>
-      </c>
       <c r="B6">
-        <v>516202</v>
+        <v>407006</v>
       </c>
       <c r="C6">
-        <v>3083</v>
+        <v>2805</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1209,74 +1138,64 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>53</v>
+        <v>45</v>
+      </c>
+      <c r="B2">
+        <v>-0.04</v>
+      </c>
+      <c r="C2">
+        <v>2.08</v>
       </c>
       <c r="D2">
-        <v>0.828</v>
-      </c>
-      <c r="E2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>0.8104</v>
+      </c>
+      <c r="E2">
+        <v>28.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" t="s">
-        <v>57</v>
+        <v>46</v>
+      </c>
+      <c r="B3">
+        <v>0.69</v>
+      </c>
+      <c r="C3">
+        <v>3.41</v>
       </c>
       <c r="D3">
-        <v>0.784</v>
-      </c>
-      <c r="E3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" t="s">
-        <v>59</v>
+        <v>0.6529</v>
+      </c>
+      <c r="E3">
+        <v>17.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>